<commit_message>
Changed the name extractor code
</commit_message>
<xml_diff>
--- a/Email_Generation_Template.xlsx
+++ b/Email_Generation_Template.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dHat\Documents\GitHub\ezeeMsgMake\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F1849A1-AA7B-4EF3-B4F5-A0B7E8953E29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B83FBCB7-51C6-47A8-8862-96857530005F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="16668" windowHeight="8748" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$2:$L$140</definedName>
@@ -28,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="261">
   <si>
     <t>First Name</t>
   </si>
@@ -66,10 +68,751 @@
     <t>Trimmed Last Name</t>
   </si>
   <si>
+    <t>Jamie</t>
+  </si>
+  <si>
     <t>FirstLast@</t>
   </si>
   <si>
-    <t>scotiabank.com</t>
+    <t>David</t>
+  </si>
+  <si>
+    <t>Lisa</t>
+  </si>
+  <si>
+    <t>Stephanie</t>
+  </si>
+  <si>
+    <t>Carlos</t>
+  </si>
+  <si>
+    <t>Curtis</t>
+  </si>
+  <si>
+    <t>Adam</t>
+  </si>
+  <si>
+    <t>Erin</t>
+  </si>
+  <si>
+    <t>Brian</t>
+  </si>
+  <si>
+    <t>Rahul</t>
+  </si>
+  <si>
+    <t>Dennis</t>
+  </si>
+  <si>
+    <t>Deanna</t>
+  </si>
+  <si>
+    <t>Nancy</t>
+  </si>
+  <si>
+    <t>Jane</t>
+  </si>
+  <si>
+    <t>Arfat</t>
+  </si>
+  <si>
+    <t>Virakti</t>
+  </si>
+  <si>
+    <t>Tomi</t>
+  </si>
+  <si>
+    <t>Rebecca</t>
+  </si>
+  <si>
+    <t>Rodney</t>
+  </si>
+  <si>
+    <t>Leaira</t>
+  </si>
+  <si>
+    <t>Michelle</t>
+  </si>
+  <si>
+    <t>Martha</t>
+  </si>
+  <si>
+    <t>Shannon</t>
+  </si>
+  <si>
+    <t>Jeff</t>
+  </si>
+  <si>
+    <t>Kirstin</t>
+  </si>
+  <si>
+    <t>Gloria</t>
+  </si>
+  <si>
+    <t>Lucas</t>
+  </si>
+  <si>
+    <t>Raylene</t>
+  </si>
+  <si>
+    <t>Leilani</t>
+  </si>
+  <si>
+    <t>Kristina</t>
+  </si>
+  <si>
+    <t>Brett</t>
+  </si>
+  <si>
+    <t>Kevin</t>
+  </si>
+  <si>
+    <t>Nina</t>
+  </si>
+  <si>
+    <t>Brianne</t>
+  </si>
+  <si>
+    <t>Nicole</t>
+  </si>
+  <si>
+    <t>Bebee</t>
+  </si>
+  <si>
+    <t>Nikki</t>
+  </si>
+  <si>
+    <t>Tanya</t>
+  </si>
+  <si>
+    <t>Mikayla</t>
+  </si>
+  <si>
+    <t>Agnes</t>
+  </si>
+  <si>
+    <t>Fiona</t>
+  </si>
+  <si>
+    <t>Susan</t>
+  </si>
+  <si>
+    <t>Connie</t>
+  </si>
+  <si>
+    <t>Elaina</t>
+  </si>
+  <si>
+    <t>Holly</t>
+  </si>
+  <si>
+    <t>Surong</t>
+  </si>
+  <si>
+    <t>Jaskirat</t>
+  </si>
+  <si>
+    <t>Chioma</t>
+  </si>
+  <si>
+    <t>Petra</t>
+  </si>
+  <si>
+    <t>Seitz</t>
+  </si>
+  <si>
+    <t>Knox</t>
+  </si>
+  <si>
+    <t>Janine</t>
+  </si>
+  <si>
+    <t>Karishma</t>
+  </si>
+  <si>
+    <t>Danna</t>
+  </si>
+  <si>
+    <t>Lauretta</t>
+  </si>
+  <si>
+    <t>Bruce</t>
+  </si>
+  <si>
+    <t>Meghan</t>
+  </si>
+  <si>
+    <t>Olanrewaju</t>
+  </si>
+  <si>
+    <t>Phil</t>
+  </si>
+  <si>
+    <t>Spencer</t>
+  </si>
+  <si>
+    <t>Angela</t>
+  </si>
+  <si>
+    <t>Becky</t>
+  </si>
+  <si>
+    <t>Bob</t>
+  </si>
+  <si>
+    <t>Laurie</t>
+  </si>
+  <si>
+    <t>Owais</t>
+  </si>
+  <si>
+    <t>Kelsey</t>
+  </si>
+  <si>
+    <t>Shelley</t>
+  </si>
+  <si>
+    <t>Lindsay</t>
+  </si>
+  <si>
+    <t>Wanda</t>
+  </si>
+  <si>
+    <t>Nichola</t>
+  </si>
+  <si>
+    <t>Blair</t>
+  </si>
+  <si>
+    <t>Mayela</t>
+  </si>
+  <si>
+    <t>Torri</t>
+  </si>
+  <si>
+    <t>Dana</t>
+  </si>
+  <si>
+    <t>Shane</t>
+  </si>
+  <si>
+    <t>Nav</t>
+  </si>
+  <si>
+    <t>Teresa</t>
+  </si>
+  <si>
+    <t>Gaurang</t>
+  </si>
+  <si>
+    <t>Wendy</t>
+  </si>
+  <si>
+    <t>Jennifer</t>
+  </si>
+  <si>
+    <t>Chelsea</t>
+  </si>
+  <si>
+    <t>Madeline</t>
+  </si>
+  <si>
+    <t>Suzy</t>
+  </si>
+  <si>
+    <t>Saqib</t>
+  </si>
+  <si>
+    <t>Shanna</t>
+  </si>
+  <si>
+    <t>Kyla</t>
+  </si>
+  <si>
+    <t>Sclina</t>
+  </si>
+  <si>
+    <t>Kathryn</t>
+  </si>
+  <si>
+    <t>Deirdra</t>
+  </si>
+  <si>
+    <t>Neil</t>
+  </si>
+  <si>
+    <t>Jacqueline</t>
+  </si>
+  <si>
+    <t>Jodi</t>
+  </si>
+  <si>
+    <t>Channing</t>
+  </si>
+  <si>
+    <t>Rupal</t>
+  </si>
+  <si>
+    <t>jane.bogatyrevich@atco.com</t>
+  </si>
+  <si>
+    <t>arfat.anwar@atco.com</t>
+  </si>
+  <si>
+    <t>virakti.anjaria@atco.com</t>
+  </si>
+  <si>
+    <t>tomi.owoyemi@atco.com</t>
+  </si>
+  <si>
+    <t>rebecca.white@atco.com</t>
+  </si>
+  <si>
+    <t>erin.jackson@atco.com</t>
+  </si>
+  <si>
+    <t>rodney.deir@atco.com</t>
+  </si>
+  <si>
+    <t>leaira.isley@atco.com</t>
+  </si>
+  <si>
+    <t>michelle.paterson@atco.com</t>
+  </si>
+  <si>
+    <t>martha.wasylynchuk@atco.com</t>
+  </si>
+  <si>
+    <t>shannon.rittmeyer@atco.com</t>
+  </si>
+  <si>
+    <t>jeff.ferguson@atco.com</t>
+  </si>
+  <si>
+    <t>kirstin.normand@atco.com</t>
+  </si>
+  <si>
+    <t>gloria.bhatia@atco.com</t>
+  </si>
+  <si>
+    <t>lucas.janke@atco.com</t>
+  </si>
+  <si>
+    <t>raylene.frehlich@atco.com</t>
+  </si>
+  <si>
+    <t>leilani.coralejo@atco.com</t>
+  </si>
+  <si>
+    <t>kristina.clayton@atco.com</t>
+  </si>
+  <si>
+    <t>brett.eigner@atco.com</t>
+  </si>
+  <si>
+    <t>kevin.lazarenko@atco.com</t>
+  </si>
+  <si>
+    <t>nina.edwards@atco.com</t>
+  </si>
+  <si>
+    <t>brianne.rainey@atco.com</t>
+  </si>
+  <si>
+    <t>nicole.maclean@atco.com</t>
+  </si>
+  <si>
+    <t>rahul.chinta@atco.com</t>
+  </si>
+  <si>
+    <t>bebee.chang@atco.com</t>
+  </si>
+  <si>
+    <t>nancy.lewis@atco.com</t>
+  </si>
+  <si>
+    <t>nikki.gjerde@atco.com</t>
+  </si>
+  <si>
+    <t>tanya.danielson@atco.com</t>
+  </si>
+  <si>
+    <t>mikayla.smetaniuk@atco.com</t>
+  </si>
+  <si>
+    <t>agnes.hickey@atco.com</t>
+  </si>
+  <si>
+    <t>fiona.broadhead@atco.com</t>
+  </si>
+  <si>
+    <t>susan.elliott@atco.com</t>
+  </si>
+  <si>
+    <t>deanna.girard@atco.com</t>
+  </si>
+  <si>
+    <t>connie.berkshire@atco.com</t>
+  </si>
+  <si>
+    <t>elaina.eifler@atco.com</t>
+  </si>
+  <si>
+    <t>holly.hutchinson@atco.com</t>
+  </si>
+  <si>
+    <t>surong.wang@atco.com</t>
+  </si>
+  <si>
+    <t>jaskirat.kalsi@atco.com</t>
+  </si>
+  <si>
+    <t>chioma.ahaneku@atco.com</t>
+  </si>
+  <si>
+    <t>petra.seitz@atco.com</t>
+  </si>
+  <si>
+    <t>knox.davidson@atco.com</t>
+  </si>
+  <si>
+    <t>janine.tornhout@atco.com</t>
+  </si>
+  <si>
+    <t>karishma.arora@atco.com</t>
+  </si>
+  <si>
+    <t>lisa.nyman@atco.com</t>
+  </si>
+  <si>
+    <t>danna.richardson@atco.com</t>
+  </si>
+  <si>
+    <t>lauretta.pearse@atco.com</t>
+  </si>
+  <si>
+    <t>bruce.legault@atco.com</t>
+  </si>
+  <si>
+    <t>meghan.stuart@atco.com</t>
+  </si>
+  <si>
+    <t>olanrewaju.oyelami@atco.com</t>
+  </si>
+  <si>
+    <t>phil.atherton@atco.com</t>
+  </si>
+  <si>
+    <t>spencer.forgo@atco.com</t>
+  </si>
+  <si>
+    <t>tanya.cake@atco.com</t>
+  </si>
+  <si>
+    <t>angela.nordstrom@atco.com</t>
+  </si>
+  <si>
+    <t>Becky.Penrice@atco.com</t>
+  </si>
+  <si>
+    <t>Brian.Bain@atco.com</t>
+  </si>
+  <si>
+    <t>Bob.Myles@atco.com</t>
+  </si>
+  <si>
+    <t>Laurie.Bos@atco.com</t>
+  </si>
+  <si>
+    <t>Owais.Khan@atco.com</t>
+  </si>
+  <si>
+    <t>Kelsey.Trovato@atco.com</t>
+  </si>
+  <si>
+    <t>Nancy.Manchak@atco.com</t>
+  </si>
+  <si>
+    <t>Jamie.Jaques@atco.com</t>
+  </si>
+  <si>
+    <t>Shelley.Faria@atco.com</t>
+  </si>
+  <si>
+    <t>Lindsay.Angelstad@atco.com</t>
+  </si>
+  <si>
+    <t>Wanda.Hulme@atco.com</t>
+  </si>
+  <si>
+    <t>Nichola.Belsheim@atco.com</t>
+  </si>
+  <si>
+    <t>Blair.Bishop@atco.com</t>
+  </si>
+  <si>
+    <t>Mayela.Neubert@atco.com</t>
+  </si>
+  <si>
+    <t>Torri.Lamash@atco.com</t>
+  </si>
+  <si>
+    <t>Dennis.Gilson@atco.com</t>
+  </si>
+  <si>
+    <t>Brett.Heath@atco.com</t>
+  </si>
+  <si>
+    <t>Dana.Johansen@atco.com</t>
+  </si>
+  <si>
+    <t>Shane.Ellis@atco.com</t>
+  </si>
+  <si>
+    <t>Nav.Basra@atco.com</t>
+  </si>
+  <si>
+    <t>Teresa.Smith@atco.com</t>
+  </si>
+  <si>
+    <t>Gaurang.Vyas@atco.com</t>
+  </si>
+  <si>
+    <t>Wendy.Armstrong@atco.com</t>
+  </si>
+  <si>
+    <t>Jennifer.Hadada@atco.com</t>
+  </si>
+  <si>
+    <t>Chelsea.Keelan@atco.com</t>
+  </si>
+  <si>
+    <t>Madeline.Dey@atco.com</t>
+  </si>
+  <si>
+    <t>David.Chiasson@atco.com</t>
+  </si>
+  <si>
+    <t>Suzy.Connolly@atco.com</t>
+  </si>
+  <si>
+    <t>Jennifer.Stinson@atco.com</t>
+  </si>
+  <si>
+    <t>David.Peterson@atco.com</t>
+  </si>
+  <si>
+    <t>Saqib.Iqbal@atco.com</t>
+  </si>
+  <si>
+    <t>Shanna.Jaap@atco.com</t>
+  </si>
+  <si>
+    <t>Adam.Wallace@atco.com</t>
+  </si>
+  <si>
+    <t>Kyla.Jenkinson@atco.com</t>
+  </si>
+  <si>
+    <t>Sclina.Lau@atco.com</t>
+  </si>
+  <si>
+    <t>Kathryn.Dickson@atco.com</t>
+  </si>
+  <si>
+    <t>Carlos.Bautista@atco.com</t>
+  </si>
+  <si>
+    <t>Deirdra.McLaughlin@atco.com</t>
+  </si>
+  <si>
+    <t>Neil.Orr@atco.com</t>
+  </si>
+  <si>
+    <t>Wendy.Chenier@atco.com</t>
+  </si>
+  <si>
+    <t>Jacqueline.Cunha@atco.com</t>
+  </si>
+  <si>
+    <t>Jodi.Collier@atco.com</t>
+  </si>
+  <si>
+    <t>Channing.Steinbring@atco.com</t>
+  </si>
+  <si>
+    <t>Rupal.Shah@atco.com</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Sarah</t>
+  </si>
+  <si>
+    <t>Sharmeen</t>
+  </si>
+  <si>
+    <t>Billy</t>
+  </si>
+  <si>
+    <t>Grey</t>
+  </si>
+  <si>
+    <t>Veronica</t>
+  </si>
+  <si>
+    <t>Tasha</t>
+  </si>
+  <si>
+    <t>Aynsley</t>
+  </si>
+  <si>
+    <t>Aashna</t>
+  </si>
+  <si>
+    <t>Cole</t>
+  </si>
+  <si>
+    <t>Samrat</t>
+  </si>
+  <si>
+    <t>Nicky</t>
+  </si>
+  <si>
+    <t>Hilda</t>
+  </si>
+  <si>
+    <t>Layla</t>
+  </si>
+  <si>
+    <t>Siobhan</t>
+  </si>
+  <si>
+    <t>Opemipo</t>
+  </si>
+  <si>
+    <t>Ankira</t>
+  </si>
+  <si>
+    <t>Karen</t>
+  </si>
+  <si>
+    <t>Ariba</t>
+  </si>
+  <si>
+    <t>canadalife.com</t>
+  </si>
+  <si>
+    <t>kevin.laljie@canadalife.com</t>
+  </si>
+  <si>
+    <t>sharmeen.malik@canadalife.com</t>
+  </si>
+  <si>
+    <t>billy.stewart@canadalife.com</t>
+  </si>
+  <si>
+    <t>grey.nutter@canadalife.com</t>
+  </si>
+  <si>
+    <t>veronica.desrosiers@canadalife.com</t>
+  </si>
+  <si>
+    <t>tasha.kokinasidis@canadalife.com</t>
+  </si>
+  <si>
+    <t>aynsley.hamilton@canadalife.com</t>
+  </si>
+  <si>
+    <t>aashna.singh@canadalife.com</t>
+  </si>
+  <si>
+    <t>cole.higgins@canadalife.com</t>
+  </si>
+  <si>
+    <t>samrat.paul@canadalife.com</t>
+  </si>
+  <si>
+    <t>nicky.leach@canadalife.com</t>
+  </si>
+  <si>
+    <t>hilda.vallapuram@canadalife.com</t>
+  </si>
+  <si>
+    <t>stephanie.anderson@canadalife.com</t>
+  </si>
+  <si>
+    <t>layla.acharoui@canadalife.com</t>
+  </si>
+  <si>
+    <t>siobhan.oneill@canadalife.com</t>
+  </si>
+  <si>
+    <t>opemipo.obaido@canadalife.com</t>
+  </si>
+  <si>
+    <t>ankira.arora@canadalife.com</t>
+  </si>
+  <si>
+    <t>nikki.vieira@canadalife.com</t>
+  </si>
+  <si>
+    <t>karen.leadbeater@canadalife.com</t>
+  </si>
+  <si>
+    <t>ariba.malik@canadalife.com</t>
+  </si>
+  <si>
+    <t>Justin</t>
+  </si>
+  <si>
+    <t>Krulicki</t>
+  </si>
+  <si>
+    <t>Reeder</t>
+  </si>
+  <si>
+    <t>Julia</t>
+  </si>
+  <si>
+    <t>Mamone</t>
+  </si>
+  <si>
+    <t>Arisha</t>
+  </si>
+  <si>
+    <t>Issani</t>
+  </si>
+  <si>
+    <t>Mohammed</t>
+  </si>
+  <si>
+    <t>Gary</t>
+  </si>
+  <si>
+    <t>Good</t>
+  </si>
+  <si>
+    <t>Chloe</t>
+  </si>
+  <si>
+    <t>McCann</t>
+  </si>
+  <si>
+    <t>Omara</t>
+  </si>
+  <si>
+    <t>Jake</t>
+  </si>
+  <si>
+    <t>Walker</t>
+  </si>
+  <si>
+    <t>Kristopher</t>
+  </si>
+  <si>
+    <t>Bates</t>
   </si>
 </sst>
 </file>
@@ -484,421 +1227,493 @@
         <v>9</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>13</v>
+        <v>223</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>244</v>
+      </c>
+      <c r="B3" t="s">
+        <v>245</v>
+      </c>
       <c r="C3" t="str">
         <f>IF(A3&lt;&gt;"",TRIM(A3),"")</f>
-        <v/>
+        <v>Justin</v>
       </c>
       <c r="D3" t="str">
         <f>IF(B3&lt;&gt;"",TRIM(B3),"")</f>
-        <v/>
+        <v>Krulicki</v>
       </c>
       <c r="E3" t="str">
         <f>IF($C3&lt;&gt;"",LOWER(CONCATENATE(LEFT($C3,1),E$1,$D3,"@",$L$2)),"")</f>
-        <v/>
+        <v>j.krulicki@canadalife.com</v>
       </c>
       <c r="F3" t="str">
         <f>IF($C3&lt;&gt;"",LOWER((CONCATENATE($C3,F$1,$D3,"@",$L$2))),"")</f>
-        <v/>
+        <v>justin.krulicki@canadalife.com</v>
       </c>
       <c r="G3" t="str">
         <f t="shared" ref="G3:H19" si="0">IF($C3&lt;&gt;"",LOWER(CONCATENATE(LEFT($C3,1),G$1,$D3,"@",$L$2)),"")</f>
-        <v/>
+        <v>jkrulicki@canadalife.com</v>
       </c>
       <c r="H3" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>j_krulicki@canadalife.com</v>
       </c>
       <c r="I3" t="str">
         <f>IF($C3&lt;&gt;"",LOWER(CONCATENATE($C3,I$1,$D3,"@",$L$2)),"")</f>
-        <v/>
+        <v>justin_krulicki@canadalife.com</v>
       </c>
       <c r="J3" t="str">
         <f>IF($C3&lt;&gt;"",LOWER(CONCATENATE($C3,J$1,$D3,"@",$L$2)),"")</f>
-        <v/>
+        <v>justinkrulicki@canadalife.com</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" t="s">
+        <v>246</v>
+      </c>
       <c r="C4" t="str">
         <f t="shared" ref="C4:C11" si="1">IF(A4&lt;&gt;"",TRIM(A4),"")</f>
-        <v/>
+        <v>Jennifer</v>
       </c>
       <c r="D4" t="str">
         <f t="shared" ref="D4:D11" si="2">IF(B4&lt;&gt;"",TRIM(B4),"")</f>
-        <v/>
+        <v>Reeder</v>
       </c>
       <c r="E4" t="str">
         <f t="shared" ref="E4:E54" si="3">IF($C4&lt;&gt;"",LOWER(CONCATENATE(LEFT($C4,1),E$1,$D4,"@",$L$2)),"")</f>
-        <v/>
+        <v>j.reeder@canadalife.com</v>
       </c>
       <c r="F4" t="str">
         <f t="shared" ref="F4:F54" si="4">IF($C4&lt;&gt;"",LOWER((CONCATENATE($C4,F$1,$D4,"@",$L$2))),"")</f>
-        <v/>
+        <v>jennifer.reeder@canadalife.com</v>
       </c>
       <c r="G4" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>jreeder@canadalife.com</v>
       </c>
       <c r="H4" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>j_reeder@canadalife.com</v>
       </c>
       <c r="I4" t="str">
         <f t="shared" ref="I4:J54" si="5">IF($C4&lt;&gt;"",LOWER(CONCATENATE($C4,I$1,$D4,"@",$L$2)),"")</f>
-        <v/>
+        <v>jennifer_reeder@canadalife.com</v>
       </c>
       <c r="J4" t="str">
         <f>IF($C4&lt;&gt;"",LOWER(CONCATENATE($C4,J$1,$D4,"@",$L$2)),"")</f>
-        <v/>
+        <v>jenniferreeder@canadalife.com</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>247</v>
+      </c>
+      <c r="B5" t="s">
+        <v>248</v>
+      </c>
       <c r="C5" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Julia</v>
       </c>
       <c r="D5" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Mamone</v>
       </c>
       <c r="E5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>j.mamone@canadalife.com</v>
       </c>
       <c r="F5" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>julia.mamone@canadalife.com</v>
       </c>
       <c r="G5" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>jmamone@canadalife.com</v>
       </c>
       <c r="H5" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>j_mamone@canadalife.com</v>
       </c>
       <c r="I5" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>julia_mamone@canadalife.com</v>
       </c>
       <c r="J5" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>juliamamone@canadalife.com</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>249</v>
+      </c>
+      <c r="B6" t="s">
+        <v>250</v>
+      </c>
       <c r="C6" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Arisha</v>
       </c>
       <c r="D6" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Issani</v>
       </c>
       <c r="E6" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>a.issani@canadalife.com</v>
       </c>
       <c r="F6" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>arisha.issani@canadalife.com</v>
       </c>
       <c r="G6" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>aissani@canadalife.com</v>
       </c>
       <c r="H6" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>a_issani@canadalife.com</v>
       </c>
       <c r="I6" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>arisha_issani@canadalife.com</v>
       </c>
       <c r="J6" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>arishaissani@canadalife.com</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>244</v>
+      </c>
+      <c r="B7" t="s">
+        <v>251</v>
+      </c>
       <c r="C7" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Justin</v>
       </c>
       <c r="D7" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Mohammed</v>
       </c>
       <c r="E7" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>j.mohammed@canadalife.com</v>
       </c>
       <c r="F7" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>justin.mohammed@canadalife.com</v>
       </c>
       <c r="G7" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>jmohammed@canadalife.com</v>
       </c>
       <c r="H7" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>j_mohammed@canadalife.com</v>
       </c>
       <c r="I7" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>justin_mohammed@canadalife.com</v>
       </c>
       <c r="J7" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>justinmohammed@canadalife.com</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>252</v>
+      </c>
+      <c r="B8" t="s">
+        <v>253</v>
+      </c>
       <c r="C8" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Gary</v>
       </c>
       <c r="D8" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Good</v>
       </c>
       <c r="E8" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>g.good@canadalife.com</v>
       </c>
       <c r="F8" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>gary.good@canadalife.com</v>
       </c>
       <c r="G8" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>ggood@canadalife.com</v>
       </c>
       <c r="H8" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>g_good@canadalife.com</v>
       </c>
       <c r="I8" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>gary_good@canadalife.com</v>
       </c>
       <c r="J8" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>garygood@canadalife.com</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
       <c r="C9" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Chelsea</v>
       </c>
       <c r="D9" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Curtis</v>
       </c>
       <c r="E9" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>c.curtis@canadalife.com</v>
       </c>
       <c r="F9" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>chelsea.curtis@canadalife.com</v>
       </c>
       <c r="G9" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>ccurtis@canadalife.com</v>
       </c>
       <c r="H9" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>c_curtis@canadalife.com</v>
       </c>
       <c r="I9" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>chelsea_curtis@canadalife.com</v>
       </c>
       <c r="J9" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>chelseacurtis@canadalife.com</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" t="s">
+        <v>62</v>
+      </c>
       <c r="C10" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Jennifer</v>
       </c>
       <c r="D10" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Seitz</v>
       </c>
       <c r="E10" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>j.seitz@canadalife.com</v>
       </c>
       <c r="F10" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>jennifer.seitz@canadalife.com</v>
       </c>
       <c r="G10" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>jseitz@canadalife.com</v>
       </c>
       <c r="H10" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>j_seitz@canadalife.com</v>
       </c>
       <c r="I10" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>jennifer_seitz@canadalife.com</v>
       </c>
       <c r="J10" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>jenniferseitz@canadalife.com</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>254</v>
+      </c>
+      <c r="B11" t="s">
+        <v>255</v>
+      </c>
       <c r="C11" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Chloe</v>
       </c>
       <c r="D11" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>McCann</v>
       </c>
       <c r="E11" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>c.mccann@canadalife.com</v>
       </c>
       <c r="F11" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>chloe.mccann@canadalife.com</v>
       </c>
       <c r="G11" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>cmccann@canadalife.com</v>
       </c>
       <c r="H11" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>c_mccann@canadalife.com</v>
       </c>
       <c r="I11" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>chloe_mccann@canadalife.com</v>
       </c>
       <c r="J11" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>chloemccann@canadalife.com</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>205</v>
+      </c>
+      <c r="B12" t="s">
+        <v>256</v>
+      </c>
       <c r="C12" t="str">
         <f>IF(A12&lt;&gt;"",TRIM(A12),"")</f>
-        <v/>
+        <v>Sarah</v>
       </c>
       <c r="D12" t="str">
         <f>IF(B12&lt;&gt;"",TRIM(B12),"")</f>
-        <v/>
+        <v>Omara</v>
       </c>
       <c r="E12" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>s.omara@canadalife.com</v>
       </c>
       <c r="F12" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>sarah.omara@canadalife.com</v>
       </c>
       <c r="G12" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>somara@canadalife.com</v>
       </c>
       <c r="H12" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>s_omara@canadalife.com</v>
       </c>
       <c r="I12" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>sarah_omara@canadalife.com</v>
       </c>
       <c r="J12" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>sarahomara@canadalife.com</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>257</v>
+      </c>
+      <c r="B13" t="s">
+        <v>258</v>
+      </c>
       <c r="C13" t="str">
         <f t="shared" ref="C13:C22" si="6">IF(A13&lt;&gt;"",TRIM(A13),"")</f>
-        <v/>
+        <v>Jake</v>
       </c>
       <c r="D13" t="str">
         <f t="shared" ref="D13:D22" si="7">IF(B13&lt;&gt;"",TRIM(B13),"")</f>
-        <v/>
+        <v>Walker</v>
       </c>
       <c r="E13" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>j.walker@canadalife.com</v>
       </c>
       <c r="F13" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>jake.walker@canadalife.com</v>
       </c>
       <c r="G13" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>jwalker@canadalife.com</v>
       </c>
       <c r="H13" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>j_walker@canadalife.com</v>
       </c>
       <c r="I13" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>jake_walker@canadalife.com</v>
       </c>
       <c r="J13" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>jakewalker@canadalife.com</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>259</v>
+      </c>
+      <c r="B14" t="s">
+        <v>260</v>
+      </c>
       <c r="C14" t="str">
         <f t="shared" si="6"/>
-        <v/>
+        <v>Kristopher</v>
       </c>
       <c r="D14" t="str">
         <f t="shared" si="7"/>
-        <v/>
+        <v>Bates</v>
       </c>
       <c r="E14" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>k.bates@canadalife.com</v>
       </c>
       <c r="F14" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>kristopher.bates@canadalife.com</v>
       </c>
       <c r="G14" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>kbates@canadalife.com</v>
       </c>
       <c r="H14" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>k_bates@canadalife.com</v>
       </c>
       <c r="I14" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>kristopher_bates@canadalife.com</v>
       </c>
       <c r="J14" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>kristopherbates@canadalife.com</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
@@ -5131,4 +5946,1763 @@
     <ignoredError sqref="F3" formula="1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48221E54-6CBD-4FAE-86C8-E398090CA7F2}">
+  <dimension ref="A1:B138"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>206</v>
+      </c>
+      <c r="B2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>208</v>
+      </c>
+      <c r="B4" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>209</v>
+      </c>
+      <c r="B5" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>210</v>
+      </c>
+      <c r="B6" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>211</v>
+      </c>
+      <c r="B7" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>212</v>
+      </c>
+      <c r="B8" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>213</v>
+      </c>
+      <c r="B9" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>214</v>
+      </c>
+      <c r="B10" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>215</v>
+      </c>
+      <c r="B11" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>216</v>
+      </c>
+      <c r="B12" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>217</v>
+      </c>
+      <c r="B14" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>218</v>
+      </c>
+      <c r="B15" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>219</v>
+      </c>
+      <c r="B16" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>220</v>
+      </c>
+      <c r="B17" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>49</v>
+      </c>
+      <c r="B18" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>221</v>
+      </c>
+      <c r="B19" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>222</v>
+      </c>
+      <c r="B20" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B21" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B22" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B23" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B24" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B25" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B26" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B27" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B28" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B29" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B30" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B31" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B32" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B33" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B34" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B35" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B36" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="37" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B37" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B38" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="39" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B39" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B40" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="41" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B41" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="42" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B42" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="43" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B43" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="44" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B44" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="45" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B45" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="46" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B46" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="47" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B47" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="48" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B48" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="49" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B49" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B50" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B51" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B52" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="53" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B53" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B54" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="55" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B55" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="56" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B56" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="57" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B57" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="58" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B58" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="59" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B59" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="60" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B60" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="61" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B61" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="62" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B62" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="63" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B63" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="64" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B64" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="65" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B65" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B66" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="67" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B67" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="68" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B68" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="69" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B69" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="70" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B70" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="71" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B71" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="72" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B72" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="73" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B73" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="74" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B74" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="75" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B75" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="76" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B76" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="77" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B77" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="78" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B78" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="79" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B79" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="80" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B80" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="81" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B81" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="82" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B82" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="83" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B83" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="84" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B84" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="85" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B85" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="86" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B86" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="87" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B87" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="88" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B88" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="89" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B89" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="90" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B90" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="91" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B91" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="92" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B92" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="93" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B93" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="94" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B94" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="95" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B95" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="96" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B96" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="97" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B97" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="98" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B98" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="99" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B99" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="100" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B100" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="101" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B101" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="102" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B102" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="103" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B103" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="104" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B104" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="105" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B105" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="106" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B106" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="107" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B107" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="108" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B108" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="109" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B109" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="110" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B110" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="111" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B111" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="112" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B112" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="113" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B113" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="114" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B114" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="115" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B115" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="116" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B116" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="117" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B117" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="118" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B118" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="119" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B119" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="120" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B120" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="121" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B121" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="122" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B122" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="123" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B123" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="124" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B124" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="125" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B125" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="126" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B126" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="127" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B127" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="128" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B128" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="129" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B129" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="130" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B130" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="131" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B131" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="132" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B132" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="133" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B133" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="134" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B134" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="135" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B135" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="136" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B136" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="137" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B137" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="138" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B138" t="s">
+        <v>204</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CBBBE82-E138-48AF-9B2B-AB1EE6ED354A}">
+  <dimension ref="A1:B139"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>38</v>
+      </c>
+      <c r="B15" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>41</v>
+      </c>
+      <c r="B18" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>46</v>
+      </c>
+      <c r="B23" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>22</v>
+      </c>
+      <c r="B25" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>48</v>
+      </c>
+      <c r="B26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>52</v>
+      </c>
+      <c r="B31" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>53</v>
+      </c>
+      <c r="B32" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>54</v>
+      </c>
+      <c r="B33" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>24</v>
+      </c>
+      <c r="B34" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>55</v>
+      </c>
+      <c r="B35" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>56</v>
+      </c>
+      <c r="B36" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>57</v>
+      </c>
+      <c r="B37" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>58</v>
+      </c>
+      <c r="B38" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>59</v>
+      </c>
+      <c r="B39" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>60</v>
+      </c>
+      <c r="B40" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>61</v>
+      </c>
+      <c r="B41" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>63</v>
+      </c>
+      <c r="B42" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>64</v>
+      </c>
+      <c r="B43" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>65</v>
+      </c>
+      <c r="B44" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>15</v>
+      </c>
+      <c r="B45" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>66</v>
+      </c>
+      <c r="B46" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>67</v>
+      </c>
+      <c r="B47" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>68</v>
+      </c>
+      <c r="B48" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>69</v>
+      </c>
+      <c r="B49" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>70</v>
+      </c>
+      <c r="B50" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>71</v>
+      </c>
+      <c r="B51" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>72</v>
+      </c>
+      <c r="B52" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>50</v>
+      </c>
+      <c r="B53" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>73</v>
+      </c>
+      <c r="B54" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>74</v>
+      </c>
+      <c r="B55" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>21</v>
+      </c>
+      <c r="B56" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>75</v>
+      </c>
+      <c r="B57" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>76</v>
+      </c>
+      <c r="B58" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>77</v>
+      </c>
+      <c r="B59" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>78</v>
+      </c>
+      <c r="B60" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>25</v>
+      </c>
+      <c r="B61" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>12</v>
+      </c>
+      <c r="B62" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>79</v>
+      </c>
+      <c r="B63" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>80</v>
+      </c>
+      <c r="B64" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>81</v>
+      </c>
+      <c r="B65" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>82</v>
+      </c>
+      <c r="B66" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>83</v>
+      </c>
+      <c r="B67" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>84</v>
+      </c>
+      <c r="B68" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>85</v>
+      </c>
+      <c r="B69" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>23</v>
+      </c>
+      <c r="B70" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>43</v>
+      </c>
+      <c r="B71" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>86</v>
+      </c>
+      <c r="B72" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>87</v>
+      </c>
+      <c r="B73" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>88</v>
+      </c>
+      <c r="B74" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>89</v>
+      </c>
+      <c r="B75" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>90</v>
+      </c>
+      <c r="B76" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>91</v>
+      </c>
+      <c r="B77" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>92</v>
+      </c>
+      <c r="B78" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>93</v>
+      </c>
+      <c r="B79" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>94</v>
+      </c>
+      <c r="B80" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>14</v>
+      </c>
+      <c r="B81" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>95</v>
+      </c>
+      <c r="B82" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>92</v>
+      </c>
+      <c r="B83" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>14</v>
+      </c>
+      <c r="B84" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>96</v>
+      </c>
+      <c r="B85" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>97</v>
+      </c>
+      <c r="B86" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>19</v>
+      </c>
+      <c r="B87" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>98</v>
+      </c>
+      <c r="B88" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>99</v>
+      </c>
+      <c r="B89" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>100</v>
+      </c>
+      <c r="B90" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>17</v>
+      </c>
+      <c r="B91" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>101</v>
+      </c>
+      <c r="B92" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>102</v>
+      </c>
+      <c r="B93" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>91</v>
+      </c>
+      <c r="B94" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
+        <v>103</v>
+      </c>
+      <c r="B95" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>104</v>
+      </c>
+      <c r="B96" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>105</v>
+      </c>
+      <c r="B97" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>106</v>
+      </c>
+      <c r="B98" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B99" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B100" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B101" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B102" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B103" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B104" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B105" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B106" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B107" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B108" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B109" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B110" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B111" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B112" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="113" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B113" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="114" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B114" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="115" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B115" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="116" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B116" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="117" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B117" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="118" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B118" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="119" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B119" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="120" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B120" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="121" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B121" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="122" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B122" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="123" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B123" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="124" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B124" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="125" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B125" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="126" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B126" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="127" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B127" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="128" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B128" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="129" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B129" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="130" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B130" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="131" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B131" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="132" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B132" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="133" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B133" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="134" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B134" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="135" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B135" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="136" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B136" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="137" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B137" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="138" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B138" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="139" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B139" t="s">
+        <v>204</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>